<commit_message>
Add support for activity sessions and enhance Excel parsing in dashboard
</commit_message>
<xml_diff>
--- a/data/AI Champions Initiative Report.xlsx
+++ b/data/AI Champions Initiative Report.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bosch-my.sharepoint.com/personal/mpi2cob_bosch_com/Documents/Boopathi Drive/BD COB AI Synergy/AI Champion Activity/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mpi2cob\Boopathi\Repository\workspace_ai_champion_tracting_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{66A33859-D096-4CB1-8915-ADADD55C98EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99CC54AF-F8B2-4486-9A18-7302BE1E5C75}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31D1963-4A05-4CD5-BFA4-5B93A7E7AD96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2E0B207-558B-4F0A-AA5E-53ABE0D8DD5B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D2E0B207-558B-4F0A-AA5E-53ABE0D8DD5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet4" sheetId="1" r:id="rId1"/>
+    <sheet name="Activity_Sessions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="70">
   <si>
     <t>Initiative Name</t>
   </si>
@@ -54,6 +55,9 @@
   </si>
   <si>
     <t>AI Champions Network</t>
+  </si>
+  <si>
+    <t>Gen AI Champions Initiative@SWD</t>
   </si>
   <si>
     <t xml:space="preserve">Acharyulu K Karthik (BD/SWD-FSB5)
@@ -144,9 +148,6 @@
     <t>Langchain, LangGraph</t>
   </si>
   <si>
-    <t>July</t>
-  </si>
-  <si>
     <t>Claude POC</t>
   </si>
   <si>
@@ -156,7 +157,7 @@
     <t>Its Available</t>
   </si>
   <si>
-    <t>Easy Info Access - All @one place</t>
+    <t>Easy Info Access - All @one place - Dashboard</t>
   </si>
   <si>
     <t>Boopathi/Nilesh</t>
@@ -172,9 +173,6 @@
     <t xml:space="preserve">Ideas Usecase - Chatbot </t>
   </si>
   <si>
-    <t>Veeresh</t>
-  </si>
-  <si>
     <t>Calendar for all AI Meets</t>
   </si>
   <si>
@@ -189,16 +187,6 @@
   <si>
     <r>
       <t xml:space="preserve">Define </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>metrics to measure AI benefits (effort savings, productivity)</t>
     </r>
     <r>
       <rPr>
@@ -207,7 +195,7 @@
         <rFont val="Aptos"/>
         <family val="2"/>
       </rPr>
-      <t>.</t>
+      <t>metrics to measure AI benefits (effort savings, productivity).</t>
     </r>
   </si>
   <si>
@@ -224,37 +212,75 @@
         <rFont val="Aptos"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> and </t>
+      <t xml:space="preserve"> and monthly global connects established.</t>
     </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t>monthly global connects</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> established.</t>
-    </r>
-  </si>
-  <si>
-    <t>Gen AI Champions Initiative@SWD</t>
+  </si>
+  <si>
+    <t>Veeresh - Nilesh</t>
+  </si>
+  <si>
+    <t>Sub Topic</t>
+  </si>
+  <si>
+    <t>Session Title</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Acharyulu K Karthik</t>
+  </si>
+  <si>
+    <t>DevDock - AI Sandbox for Bosch Developers</t>
+  </si>
+  <si>
+    <t>Building AI-Powered Applications with Spring MCP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murugaboopathi </t>
+  </si>
+  <si>
+    <t>Sivasankar &amp; Sivasubramanian</t>
+  </si>
+  <si>
+    <t>A2A Protocol in Action: Agent Communication and Workflow Orchestration</t>
+  </si>
+  <si>
+    <t>Upcoming</t>
+  </si>
+  <si>
+    <t>Srilakshmy Sooraj</t>
+  </si>
+  <si>
+    <t>Completion Date</t>
+  </si>
+  <si>
+    <t>Pilot Testing V1</t>
+  </si>
+  <si>
+    <t>V2 Testing</t>
+  </si>
+  <si>
+    <t>https://inside-docupedia.bosch.com/confluence/display/IGPMMCR/System+architecture</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -318,9 +344,25 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Verdana"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Aptos"/>
       <family val="2"/>
     </font>
@@ -357,7 +399,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -559,21 +601,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -597,6 +624,121 @@
       </right>
       <top/>
       <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -605,7 +747,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -655,17 +797,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -681,21 +821,61 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1036,192 +1216,199 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.33203125" customWidth="1"/>
+    <col min="2" max="2" width="46.109375" customWidth="1"/>
     <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="37.5546875" customWidth="1"/>
     <col min="5" max="5" width="34.44140625" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" customWidth="1"/>
-    <col min="7" max="7" width="10.88671875" customWidth="1"/>
-    <col min="8" max="8" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="E1" s="29" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
-        <v>51</v>
+      <c r="A2" s="57" t="s">
+        <v>5</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="38"/>
+      <c r="A3" s="57"/>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="38"/>
+      <c r="A4" s="57"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="38"/>
+      <c r="A5" s="57"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="38"/>
+      <c r="A6" s="57"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="39"/>
+      <c r="A7" s="58"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="12">
         <f>AVERAGE(C11:C25)</f>
-        <v>0.37142857142857144</v>
+        <v>0.38750000000000001</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="14"/>
+      <c r="F10" s="13"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="15"/>
       <c r="B11" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" s="17">
         <v>0.5</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="19" t="s">
         <v>27</v>
+      </c>
+      <c r="E11" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="59">
+        <v>46387</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="15"/>
       <c r="B12" s="16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" s="17">
         <v>0.5</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>29</v>
+        <v>27</v>
+      </c>
+      <c r="E12" s="45" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="59">
+        <v>46326</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="15"/>
       <c r="B13" s="16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C13" s="17">
         <v>0.5</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13" s="19"/>
+        <v>32</v>
+      </c>
+      <c r="E13" s="45"/>
+      <c r="F13" s="18"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
       <c r="B14" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C14" s="17"/>
       <c r="D14" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="45" t="s">
         <v>34</v>
       </c>
+      <c r="F14" s="18"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="15"/>
@@ -1230,138 +1417,309 @@
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="19"/>
+        <v>11</v>
+      </c>
+      <c r="E15" s="45"/>
+      <c r="F15" s="59"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="15"/>
       <c r="B16" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="32">
         <v>1</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" s="37" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="45" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F16" s="59">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="15"/>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="17"/>
+      <c r="C17" s="17">
+        <v>0.5</v>
+      </c>
       <c r="D17" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="19"/>
-    </row>
-    <row r="18" spans="1:5" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="15"/>
-      <c r="B18" s="35" t="s">
+      <c r="E17" s="45"/>
+      <c r="F17" s="59">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="27.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="33"/>
+      <c r="B18" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18" t="s">
+      <c r="C18" s="35"/>
+      <c r="D18" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="19"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16" t="s">
+      <c r="E18" s="46"/>
+      <c r="F18" s="18"/>
+    </row>
+    <row r="19" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="41"/>
+      <c r="B19" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="18" t="s">
+      <c r="C19" s="43"/>
+      <c r="D19" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="47"/>
+      <c r="F19" s="21"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="37"/>
+      <c r="B20" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="19"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="15"/>
-      <c r="B20" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E20" s="19"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C20" s="39"/>
+      <c r="D20" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" s="48"/>
+      <c r="F20" s="21"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="15"/>
       <c r="B21" s="16"/>
       <c r="C21" s="17"/>
       <c r="D21" s="18"/>
-      <c r="E21" s="19"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E21" s="45"/>
+      <c r="F21" s="21"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="15"/>
-      <c r="B22" s="20" t="s">
-        <v>45</v>
+      <c r="B22" s="19" t="s">
+        <v>44</v>
       </c>
       <c r="C22" s="17">
         <v>0</v>
       </c>
       <c r="D22" s="18"/>
-      <c r="E22" s="19"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E22" s="45"/>
+      <c r="F22" s="21"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="15"/>
-      <c r="B23" s="20" t="s">
-        <v>46</v>
+      <c r="B23" s="19" t="s">
+        <v>45</v>
       </c>
       <c r="C23" s="17">
         <v>0.1</v>
       </c>
       <c r="D23" s="18"/>
-      <c r="E23" s="19"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="21"/>
-      <c r="B24" s="20" t="s">
-        <v>47</v>
+      <c r="E23" s="45"/>
+      <c r="F23" s="21"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="20"/>
+      <c r="B24" s="19" t="s">
+        <v>46</v>
       </c>
       <c r="C24" s="17">
         <v>0</v>
       </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="19"/>
-    </row>
-    <row r="25" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="23"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="27"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B26" s="32"/>
-    </row>
-    <row r="27" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B27" s="33" t="s">
+      <c r="D24" s="21"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="21"/>
+    </row>
+    <row r="25" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="22"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="30"/>
+    </row>
+    <row r="27" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B27" s="52" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="21.6" x14ac:dyDescent="0.3">
+      <c r="B28" s="52" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="B28" s="33" t="s">
+    <row r="29" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B29" s="52" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B29" s="33" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:A7"/>
   </mergeCells>
+  <phoneticPr fontId="9" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B801DB02-CDD2-44D6-A509-9412FED4CA72}">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.6640625" customWidth="1"/>
+    <col min="2" max="2" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.77734375" style="51" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="67.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="53">
+        <v>46183</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" s="54" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="53">
+        <v>46206</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="55" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="53"/>
+      <c r="D4" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="56" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="55" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="21"/>
+      <c r="D5" s="55" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="55" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="21"/>
+      <c r="D6" s="55" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="21"/>
+      <c r="B7" s="55"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="55"/>
+      <c r="E7" s="21"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="21"/>
+      <c r="B8" s="55"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="21"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="21"/>
+      <c r="B9" s="55"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="55"/>
+      <c r="E9" s="21"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{54FEFA70-E4B4-4C12-81BB-70B5E8D78EF0}">
+      <formula1>46023</formula1>
+      <formula2>46387</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{9211E590-0678-4575-A91A-CB6F8551BFC9}">
+      <formula1>"Upcoming, Completed"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Implement Excel parsing and SharePoint integration for AI Champions Initiative dashboard
- Added `excel_parser.py` to parse the Gen AI Champions Initiative Excel sheet into structured data, handling various regions and optional child records.
- Introduced `sharepoint_sync.py` to download the tracking Excel file from SharePoint/OneDrive using Azure AD app registration, supporting both shared link and direct site path modes.
- Updated `README.md` to reflect changes in the Streamlit run URL.
- Enhanced `app.py` to integrate an AI chat assistant using LLM, allowing users to query initiative data.
- Added `description steps.txt` for user guidance on downloading files and configuring SharePoint.
- Removed deprecated `llm_client.py` and `models.py` as their functionality is now integrated into `app.py`.
- Updated `requirements.txt` to include new dependencies for requests and Office365 client.
</commit_message>
<xml_diff>
--- a/data/AI Champions Initiative Report.xlsx
+++ b/data/AI Champions Initiative Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mpi2cob\Boopathi\Repository\workspace_ai_champion_tracting_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31D1963-4A05-4CD5-BFA4-5B93A7E7AD96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B38B328-ADE1-4DA3-A305-174F6FC4471C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D2E0B207-558B-4F0A-AA5E-53ABE0D8DD5B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2E0B207-558B-4F0A-AA5E-53ABE0D8DD5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet4" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="72">
   <si>
     <t>Initiative Name</t>
   </si>
@@ -157,16 +157,9 @@
     <t>Its Available</t>
   </si>
   <si>
-    <t>Easy Info Access - All @one place - Dashboard</t>
-  </si>
-  <si>
     <t>Boopathi/Nilesh</t>
   </si>
   <si>
-    <t>Repository - Capture the information - AI topics 
-Gen AI Stories</t>
-  </si>
-  <si>
     <t>Shanthi</t>
   </si>
   <si>
@@ -183,6 +176,75 @@
   </si>
   <si>
     <t>Gen AI News Letter @SWD</t>
+  </si>
+  <si>
+    <t>Create a central tracking mechanism (Excel → dashboard/Power BI/JIRA) for all AI activities.</t>
+  </si>
+  <si>
+    <t>Veeresh - Nilesh</t>
+  </si>
+  <si>
+    <t>Sub Topic</t>
+  </si>
+  <si>
+    <t>Session Title</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Acharyulu K Karthik</t>
+  </si>
+  <si>
+    <t>DevDock - AI Sandbox for Bosch Developers</t>
+  </si>
+  <si>
+    <t>Building AI-Powered Applications with Spring MCP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murugaboopathi </t>
+  </si>
+  <si>
+    <t>Sivasankar &amp; Sivasubramanian</t>
+  </si>
+  <si>
+    <t>A2A Protocol in Action: Agent Communication and Workflow Orchestration</t>
+  </si>
+  <si>
+    <t>Upcoming</t>
+  </si>
+  <si>
+    <t>Srilakshmy Sooraj</t>
+  </si>
+  <si>
+    <t>Completion Date</t>
+  </si>
+  <si>
+    <t>Pilot Testing V1</t>
+  </si>
+  <si>
+    <t>V2 Testing</t>
+  </si>
+  <si>
+    <t>https://inside-docupedia.bosch.com/confluence/display/IGPMMCR/System+architecture</t>
+  </si>
+  <si>
+    <t>Phase 2 updates are in-progress</t>
+  </si>
+  <si>
+    <t>Repriortization is going on</t>
   </si>
   <si>
     <r>
@@ -191,15 +253,12 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos"/>
         <family val="2"/>
       </rPr>
       <t>metrics to measure AI benefits (effort savings, productivity).</t>
     </r>
-  </si>
-  <si>
-    <t>Create a central tracking mechanism (Excel → dashboard/Power BI/JIRA) for all AI activities.</t>
   </si>
   <si>
     <r>
@@ -208,7 +267,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos"/>
         <family val="2"/>
       </rPr>
@@ -216,71 +275,17 @@
     </r>
   </si>
   <si>
-    <t>Veeresh - Nilesh</t>
-  </si>
-  <si>
-    <t>Sub Topic</t>
-  </si>
-  <si>
-    <t>Session Title</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Owner</t>
-  </si>
-  <si>
-    <t>Link</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>Acharyulu K Karthik</t>
-  </si>
-  <si>
-    <t>DevDock - AI Sandbox for Bosch Developers</t>
-  </si>
-  <si>
-    <t>Building AI-Powered Applications with Spring MCP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Murugaboopathi </t>
-  </si>
-  <si>
-    <t>Sivasankar &amp; Sivasubramanian</t>
-  </si>
-  <si>
-    <t>A2A Protocol in Action: Agent Communication and Workflow Orchestration</t>
-  </si>
-  <si>
-    <t>Upcoming</t>
-  </si>
-  <si>
-    <t>Srilakshmy Sooraj</t>
-  </si>
-  <si>
-    <t>Completion Date</t>
-  </si>
-  <si>
-    <t>Pilot Testing V1</t>
-  </si>
-  <si>
-    <t>V2 Testing</t>
-  </si>
-  <si>
-    <t>https://inside-docupedia.bosch.com/confluence/display/IGPMMCR/System+architecture</t>
+    <t>Repository - Capture the information - AI topics Gen AI Stories</t>
+  </si>
+  <si>
+    <t>Collect input from the team on the feedback of Claude, Get the information from central team as well</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -338,21 +343,10 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Verdana"/>
     </font>
     <font>
       <sz val="11"/>
@@ -365,6 +359,26 @@
       <color rgb="FF000000"/>
       <name val="Aptos"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -399,7 +413,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -601,21 +615,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -635,45 +634,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -738,6 +698,19 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -747,7 +720,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -792,20 +765,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -818,65 +781,120 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1212,7 +1230,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{651BC675-1C9F-41FC-B0E3-8041898084B3}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
@@ -1224,24 +1242,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="29" t="s">
+      <c r="E1" s="21" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="75" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="1"/>
@@ -1254,7 +1272,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="57"/>
+      <c r="A3" s="75"/>
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1269,7 +1287,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="57"/>
+      <c r="A4" s="75"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="2" t="s">
@@ -1280,7 +1298,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="57"/>
+      <c r="A5" s="75"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="2" t="s">
@@ -1291,7 +1309,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="57"/>
+      <c r="A6" s="75"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2" t="s">
@@ -1302,7 +1320,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="58"/>
+      <c r="A7" s="76"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="5" t="s">
@@ -1330,7 +1348,7 @@
         <v>24</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1340,7 +1358,7 @@
       <c r="B10" s="11"/>
       <c r="C10" s="12">
         <f>AVERAGE(C11:C25)</f>
-        <v>0.38750000000000001</v>
+        <v>0.48571428571428571</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="14"/>
@@ -1348,225 +1366,288 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="15"/>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="29">
         <v>0.5</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="45" t="s">
+      <c r="E11" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="59">
+      <c r="F11" s="27">
         <v>46387</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="15"/>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="62" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="64">
         <v>0.5</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="58" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="45" t="s">
+      <c r="E12" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="59">
-        <v>46326</v>
-      </c>
+      <c r="F12" s="27"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="15"/>
-      <c r="B13" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="17">
-        <v>0.5</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="45"/>
-      <c r="F13" s="18"/>
+      <c r="B13" s="63"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="66"/>
+      <c r="E13" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="F13" s="16"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
-      <c r="B14" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="F14" s="18"/>
+      <c r="B14" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="29">
+        <v>0.5</v>
+      </c>
+      <c r="D14" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14" s="16"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="15"/>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="35"/>
+      <c r="D15" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="27"/>
+    </row>
+    <row r="16" spans="1:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="15"/>
+      <c r="B16" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="18" t="s">
+      <c r="C16" s="69"/>
+      <c r="D16" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="45"/>
-      <c r="F15" s="59"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="15"/>
-      <c r="B16" s="16" t="s">
+      <c r="E16" s="79" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="77">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="15"/>
+      <c r="B17" s="68"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="72"/>
+      <c r="E17" s="80"/>
+      <c r="F17" s="78"/>
+    </row>
+    <row r="18" spans="1:6" ht="27.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="15"/>
+      <c r="B18" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C18" s="36">
         <v>1</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D18" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="45" t="s">
+      <c r="E18" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="F16" s="59">
-        <v>46233</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="15"/>
-      <c r="B17" s="31" t="s">
+      <c r="F18" s="16"/>
+    </row>
+    <row r="19" spans="1:6" ht="21.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="15"/>
+      <c r="B19" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="29">
+        <v>0.8</v>
+      </c>
+      <c r="D19" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="17">
-        <v>0.5</v>
-      </c>
-      <c r="D17" s="18" t="s">
+      <c r="E19" s="31"/>
+      <c r="F19" s="17"/>
+    </row>
+    <row r="20" spans="1:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="15"/>
+      <c r="B20" s="73" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="56"/>
+      <c r="D20" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="45"/>
-      <c r="F17" s="59">
-        <v>46265</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="27.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="33"/>
-      <c r="B18" s="34" t="s">
+      <c r="E20" s="60"/>
+      <c r="F20" s="17"/>
+    </row>
+    <row r="21" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="15"/>
+      <c r="B21" s="74"/>
+      <c r="C21" s="57"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="61"/>
+      <c r="F21" s="17"/>
+    </row>
+    <row r="22" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="15"/>
+      <c r="B22" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="46"/>
-      <c r="F18" s="18"/>
-    </row>
-    <row r="19" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="41"/>
-      <c r="B19" s="42" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19" s="43"/>
-      <c r="D19" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="E19" s="47"/>
-      <c r="F19" s="21"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="37"/>
-      <c r="B20" s="38" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="39"/>
-      <c r="D20" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="E20" s="48"/>
-      <c r="F20" s="21"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="15"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="21"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="15"/>
-      <c r="B22" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="17">
-        <v>0</v>
-      </c>
-      <c r="D22" s="18"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="21"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" s="42"/>
+      <c r="F22" s="17"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="15"/>
-      <c r="B23" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="C23" s="17">
+      <c r="B23" s="43" t="s">
+        <v>41</v>
+      </c>
+      <c r="C23" s="44"/>
+      <c r="D23" s="45" t="s">
+        <v>32</v>
+      </c>
+      <c r="E23" s="46"/>
+      <c r="F23" s="17"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="15"/>
+      <c r="B24" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="29">
+        <v>0</v>
+      </c>
+      <c r="D24" s="30"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="17"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="15"/>
+      <c r="B25" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="29">
         <v>0.1</v>
       </c>
-      <c r="D23" s="18"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="21"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="20"/>
-      <c r="B24" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="17">
+      <c r="D25" s="30"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="17"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="15"/>
+      <c r="B26" s="35" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="29">
         <v>0</v>
       </c>
-      <c r="D24" s="21"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="21"/>
-    </row>
-    <row r="25" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="22"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="30"/>
+      <c r="D26" s="50"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="17"/>
     </row>
     <row r="27" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B27" s="52" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="B28" s="52" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B29" s="52" t="s">
-        <v>49</v>
-      </c>
+      <c r="A27" s="15"/>
+      <c r="B27" s="51" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" s="32">
+        <v>0</v>
+      </c>
+      <c r="D27" s="47"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="17"/>
+    </row>
+    <row r="28" spans="1:6" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="15"/>
+      <c r="B28" s="51" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="55">
+        <v>0</v>
+      </c>
+      <c r="D28" s="52"/>
+      <c r="E28" s="53"/>
+      <c r="F28" s="17"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="15"/>
+      <c r="B29" s="48"/>
+      <c r="C29" s="49"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="15"/>
+      <c r="B30" s="48"/>
+      <c r="C30" s="49"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="15"/>
+      <c r="B31" s="48"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="15"/>
+      <c r="B32" s="48"/>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B33" s="48"/>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B34" s="48"/>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B35" s="48"/>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B36" s="48"/>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B37" s="48"/>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B38" s="48"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="12">
     <mergeCell ref="A2:A7"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B20:B21"/>
   </mergeCells>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1578,7 +1659,7 @@
   <cols>
     <col min="1" max="1" width="27.6640625" customWidth="1"/>
     <col min="2" max="2" width="41.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.77734375" style="51" customWidth="1"/>
+    <col min="3" max="3" width="29.77734375" style="23" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="28.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="67.109375" customWidth="1"/>
@@ -1586,137 +1667,139 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="50" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="54">
+        <v>46183</v>
+      </c>
+      <c r="D2" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E2" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="54">
+        <v>46206</v>
+      </c>
+      <c r="D3" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" s="54">
+        <v>46230</v>
+      </c>
+      <c r="D4" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="17"/>
+      <c r="D5" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="21" t="s">
+      <c r="F5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="53">
-        <v>46183</v>
-      </c>
-      <c r="D2" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="E2" s="54" t="s">
-        <v>62</v>
-      </c>
-      <c r="F2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" s="53">
-        <v>46206</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="55" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" s="53"/>
-      <c r="D4" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="E4" s="56" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="55" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="55" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="F5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="55" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="21"/>
-      <c r="D6" s="55" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>58</v>
+      <c r="E6" s="17" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="21"/>
-      <c r="B7" s="55"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="21"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="17"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="21"/>
-      <c r="B8" s="55"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="55"/>
-      <c r="E8" s="21"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="17"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="21"/>
-      <c r="B9" s="55"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="21"/>
+      <c r="A9" s="17"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="17"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{54FEFA70-E4B4-4C12-81BB-70B5E8D78EF0}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 C5:C1048576" xr:uid="{54FEFA70-E4B4-4C12-81BB-70B5E8D78EF0}">
       <formula1>46023</formula1>
       <formula2>46387</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{9211E590-0678-4575-A91A-CB6F8551BFC9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1 D5:D1048576" xr:uid="{9211E590-0678-4575-A91A-CB6F8551BFC9}">
       <formula1>"Upcoming, Completed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>